<commit_message>
Harden 1-row schema fixtures with data band and RowData rules.
Add data cells to schema_header_1row, validate RowData keys and disallow single-row header merges, add empty-header-valid pass case, drop table_schema goldens for error cases, and document planned schema test trees.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/schema_header_1row/1-row-empty-header/workbook.xlsx
+++ b/excel/testdata/schema_header_1row/1-row-empty-header/workbook.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>headerA</t>
   </si>
@@ -23,6 +23,42 @@
   </si>
   <si>
     <t>headerC</t>
+  </si>
+  <si>
+    <t>r2cA</t>
+  </si>
+  <si>
+    <t>r3cA</t>
+  </si>
+  <si>
+    <t>r4cA</t>
+  </si>
+  <si>
+    <t>r2cB</t>
+  </si>
+  <si>
+    <t>r3cB</t>
+  </si>
+  <si>
+    <t>r4cB</t>
+  </si>
+  <si>
+    <t>r2cC</t>
+  </si>
+  <si>
+    <t>r3cC</t>
+  </si>
+  <si>
+    <t>r4cC</t>
+  </si>
+  <si>
+    <t>r2cD</t>
+  </si>
+  <si>
+    <t>r3cD</t>
+  </si>
+  <si>
+    <t>r4cD</t>
   </si>
 </sst>
 </file>
@@ -340,6 +376,48 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>